<commit_message>
fix: correct DQ scorecard PASS/OPEN classification and audit data values
- Fixed 13 defects incorrectly marked OPEN with Affected_Rows=0
  - 11 rules are clean (data quality passed) -> marked Status=PASS
  - DQ-011 (phone format): 10,200 records store 91-prefixed 12-digit
    numbers instead of 10-digit Indian mobile -> OPEN, rows updated
  - DQ-012 (KYC_Status vocab): 9,035 records use 'Completed' instead
    of approved 'Verified' -> OPEN, rows updated
- Updated all Business_Impact text for PASS rules
- Updated DQ KPI Summary: 18 real defects (was 16), 11 PASS rules
- Added Methodology sheet to customer_360_summary.xlsx documenting
  Risk Index 0-100 scale and OD-facility negative balance explanation
- Updated Executive Presentation PPTX (deck_builder.py fix)
</commit_message>
<xml_diff>
--- a/output/customer_360_summary.xlsx
+++ b/output/customer_360_summary.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Summary" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Digital Summary" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,9 +24,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -56,9 +56,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -973,25 +974,24 @@
       <c r="B5" t="n">
         <v>10200</v>
       </c>
-      <c r="C5" s="1" t="n">
-        <v>46085.37715686274</v>
-      </c>
-      <c r="D5" s="1" t="n">
+      <c r="C5" s="2" t="n">
+        <v>46085.37715686343</v>
+      </c>
+      <c r="D5" s="2" t="n">
         <v>44460</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>46026</v>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="F5" s="2" t="n">
         <v>46145</v>
       </c>
-      <c r="G5" s="1" t="n">
+      <c r="G5" s="2" t="n">
         <v>46207</v>
       </c>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="2" t="n">
         <v>46248</v>
       </c>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1852,25 +1852,24 @@
       <c r="B3" t="n">
         <v>10200</v>
       </c>
-      <c r="C3" s="1" t="n">
-        <v>46158.67058823529</v>
-      </c>
-      <c r="D3" s="1" t="n">
+      <c r="C3" s="2" t="n">
+        <v>46158.67058824074</v>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>45389</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>46124</v>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="F3" s="2" t="n">
         <v>46186</v>
       </c>
-      <c r="G3" s="1" t="n">
+      <c r="G3" s="2" t="n">
         <v>46223</v>
       </c>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>46248</v>
       </c>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2176,4 +2175,66 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Silent_Churn_Risk_Index</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Weighted composite score 0-100 (higher = greater churn risk). NOT 0-1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Risk_Band</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Low (&lt;30), Moderate (30-50), High (50-65), Very High (&gt;65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Total_Balance</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Includes overdraft accounts (negative balance is valid for OD facility holders)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>